<commit_message>
rebuild work with audio files
</commit_message>
<xml_diff>
--- a/Docs/WhatINeed.xlsx
+++ b/Docs/WhatINeed.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21029"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E2E8D20-E99C-4B6D-8425-ABCAA5DE9A17}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{530EBF3B-48D4-4B8F-B46B-860B8C8D26F3}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
   <si>
     <t>Что нужно</t>
   </si>
@@ -161,6 +161,27 @@
   </si>
   <si>
     <t>сделай работу с боями переборами</t>
+  </si>
+  <si>
+    <t>отображение и обновление песен</t>
+  </si>
+  <si>
+    <t>добавить аудио для аккордов</t>
+  </si>
+  <si>
+    <t>протестировать подписки и уведомления</t>
+  </si>
+  <si>
+    <t>добавить ии для генерации текста</t>
+  </si>
+  <si>
+    <t>подвести counts для патернов и аккордов</t>
+  </si>
+  <si>
+    <t>реализовать удаление из бд как удаление из песен</t>
+  </si>
+  <si>
+    <t>сделано</t>
   </si>
 </sst>
 </file>
@@ -777,10 +798,10 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="8" t="s">
         <v>19</v>
       </c>
     </row>
@@ -789,10 +810,10 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="8" t="s">
         <v>22</v>
       </c>
     </row>
@@ -801,10 +822,10 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="8" t="s">
         <v>42</v>
       </c>
     </row>
@@ -813,10 +834,10 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="8" t="s">
         <v>32</v>
       </c>
     </row>
@@ -828,7 +849,9 @@
       <c r="C17" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="8"/>
+      <c r="D17" s="8" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B18" s="12">
@@ -838,7 +861,9 @@
       <c r="C18" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="8"/>
+      <c r="D18" s="8" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B19" s="12">
@@ -848,7 +873,9 @@
       <c r="C19" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="8"/>
+      <c r="D19" s="8" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B20" s="12">
@@ -858,7 +885,9 @@
       <c r="C20" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D20" s="8"/>
+      <c r="D20" s="8" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B21" s="12">
@@ -868,7 +897,9 @@
       <c r="C21" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="8"/>
+      <c r="D21" s="8" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B22" s="12">
@@ -895,36 +926,60 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
+      <c r="C24" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" s="2"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B25" s="12">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
+      <c r="C25" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D25" s="2"/>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B26" s="12">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
+      <c r="C26" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" s="2"/>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B27" s="12">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
+      <c r="C27" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" s="2"/>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B28" s="12">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
+      <c r="C28" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D28" s="2"/>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B29" s="12">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
+      <c r="C29" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D29" s="2"/>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B30" s="12">

</xml_diff>